<commit_message>
Fondos: cada cuerpo colegiado es de un fondo, y sus actas con él
Corrige lo anterior, que entendió «programa o proyecto» como una etiqueta
por acta. Lo que organiza las actas es el fondo: el FAP tiene su Junta
Administrativa, y lo que ella resuelve es del FAP.

- La hoja Programas pasa a ser Fondos (FIAS, FAP, FEIG y los demás fondos,
  programas o proyectos que administre el FIAS). La columna «Fondo» de
  Cuerpos dice de cuál es cada cuerpo; actas y resoluciones lo heredan.
  Se quitan las columnas de programa de Actas y Resoluciones.
- Todas las actas siguen en una sola hoja. En la página, una barra arriba
  del panel y de cada listado elige un fondo o todos, y el panel trae una
  tarjeta por fondo.
- La norma lleva su fondo o, vacío, el de su órgano.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FkuX6y6rjtHhRzfZ7rBQRg
</commit_message>
<xml_diff>
--- a/demo/matriz_demo.xlsx
+++ b/demo/matriz_demo.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuerpos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fondos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuerpos" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actas" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resoluciones" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Normativa" sheetId="6" state="visible" r:id="rId6"/>
@@ -184,22 +184,17 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Corta y sin repetirse (p. ej. JA-FAP). Es como se escribe el cuerpo en las demás hojas.</t>
+        <t>Corta y sin repetirse: FIAS, FAP, FEIG… Es como se escribe el fondo en las hojas Cuerpos y Normativa.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Como debe leerse en pantalla: «Junta Administrativa del FAP».</t>
+        <t>Como debe leerse en pantalla.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>FIAS, FAP o FEIG.</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>Qué frase abre las actas y resoluciones de este cuerpo. Si todos los abogados ven todo, deja «legal» en todas las filas.</t>
+        <t>Institución, Fondo, Programa o Proyecto.</t>
       </text>
     </comment>
   </commentList>
@@ -214,17 +209,22 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Sin repetirse. Es como se escribe en las hojas Actas y Resoluciones.</t>
+        <t>Corta y sin repetirse (p. ej. JA-FAP). Es como se escribe el cuerpo en las demás hojas.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Programa o Proyecto.</t>
+        <t>Como debe leerse en pantalla: «Junta Administrativa del FAP».</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>FIAS, FAP o FEIG.</t>
+        <t>De qué fondo, programa o proyecto es este cuerpo (sigla de la hoja Fondos). Sus actas y resoluciones se ven bajo ese fondo: la Junta Administrativa del FAP es del FAP.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Qué frase abre las actas y resoluciones de este cuerpo. Si todos los abogados ven todo, deja «legal» en todas las filas.</t>
       </text>
     </comment>
   </commentList>
@@ -259,20 +259,15 @@
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>De cuál trata la sesión (como está en la hoja Programas). Si trata de varios, sepáralos con punto y coma. Vacío = asunto general.</t>
+        <t>Enlace al PDF en la carpeta. Opcional.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Enlace al PDF en la carpeta. Opcional.</t>
+        <t>Enlace al PDF firmado. Mientras esté vacío, el acta se muestra como provisional.</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>Enlace al PDF firmado. Mientras esté vacío, el acta se muestra como provisional.</t>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <t>Cuándo se aprobó el acta definitiva (normalmente, en la sesión siguiente).</t>
       </text>
@@ -314,11 +309,6 @@
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Por omisión, la resolución es del programa o proyecto de su acta. Escríbelo aquí solo si esta resolución trata de otro, o de uno solo entre varios. Varios: separados con punto y coma.</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
         <t>Si la resolución tiene documento propio (certificación, extracto).</t>
       </text>
     </comment>
@@ -344,7 +334,7 @@
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>FIAS, FAP o FEIG.</t>
+        <t>De qué fondo es la norma (sigla de la hoja Fondos). Vacío = el fondo del órgano que la aprueba.</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
@@ -427,12 +417,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tCuerpos" displayName="tCuerpos" ref="A1:E4" headerRowCount="1">
-  <autoFilter ref="A1:E4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tFondos" displayName="tFondos" ref="A1:D5" headerRowCount="1">
+  <autoFilter ref="A1:D5"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Sigla"/>
+    <tableColumn id="2" name="Nombre completo"/>
+    <tableColumn id="3" name="Tipo"/>
+    <tableColumn id="4" name="Observaciones"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tCuerpos" displayName="tCuerpos" ref="A1:E5" headerRowCount="1">
+  <autoFilter ref="A1:E5"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Sigla"/>
     <tableColumn id="2" name="Nombre completo"/>
-    <tableColumn id="3" name="Entidad"/>
+    <tableColumn id="3" name="Fondo"/>
     <tableColumn id="4" name="Grupo de acceso"/>
     <tableColumn id="5" name="Observaciones"/>
   </tableColumns>
@@ -440,49 +443,34 @@
 </table>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tProgramas" displayName="tProgramas" ref="A1:D4" headerRowCount="1">
-  <autoFilter ref="A1:D4"/>
-  <tableColumns count="4">
-    <tableColumn id="1" name="Programa o proyecto"/>
-    <tableColumn id="2" name="Tipo"/>
-    <tableColumn id="3" name="Entidad"/>
-    <tableColumn id="4" name="Observaciones"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
-</table>
-</file>
-
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tActas" displayName="tActas" ref="A1:I26" headerRowCount="1">
-  <autoFilter ref="A1:I26"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tActas" displayName="tActas" ref="A1:H28" headerRowCount="1">
+  <autoFilter ref="A1:H28"/>
+  <tableColumns count="8">
     <tableColumn id="1" name="Cuerpo colegiado"/>
     <tableColumn id="2" name="Fecha de la sesión"/>
     <tableColumn id="3" name="Tipo de sesión"/>
     <tableColumn id="4" name="N.º de sesión"/>
-    <tableColumn id="5" name="Programa o proyecto"/>
-    <tableColumn id="6" name="Acta provisional (enlace)"/>
-    <tableColumn id="7" name="Acta definitiva (enlace)"/>
-    <tableColumn id="8" name="Fecha de aprobación del acta definitiva"/>
-    <tableColumn id="9" name="Observaciones"/>
+    <tableColumn id="5" name="Acta provisional (enlace)"/>
+    <tableColumn id="6" name="Acta definitiva (enlace)"/>
+    <tableColumn id="7" name="Fecha de aprobación del acta definitiva"/>
+    <tableColumn id="8" name="Observaciones"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tResoluciones" displayName="tResoluciones" ref="A1:H57" headerRowCount="1">
-  <autoFilter ref="A1:H57"/>
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tResoluciones" displayName="tResoluciones" ref="A1:G60" headerRowCount="1">
+  <autoFilter ref="A1:G60"/>
+  <tableColumns count="7">
     <tableColumn id="1" name="Cuerpo colegiado"/>
     <tableColumn id="2" name="Fecha de la sesión"/>
     <tableColumn id="3" name="Punto del orden del día"/>
     <tableColumn id="4" name="Lo que se resolvió"/>
     <tableColumn id="5" name="Materia"/>
-    <tableColumn id="6" name="Programa o proyecto (solo si es distinto del acta)"/>
-    <tableColumn id="7" name="Enlace (opcional)"/>
-    <tableColumn id="8" name="Observaciones"/>
+    <tableColumn id="6" name="Enlace (opcional)"/>
+    <tableColumn id="7" name="Observaciones"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
 </table>
@@ -494,7 +482,7 @@
   <tableColumns count="9">
     <tableColumn id="1" name="Nombre de la norma"/>
     <tableColumn id="2" name="Tipo"/>
-    <tableColumn id="3" name="Entidad"/>
+    <tableColumn id="3" name="Fondo"/>
     <tableColumn id="4" name="Órgano que la aprueba"/>
     <tableColumn id="5" name="Fecha de aprobación"/>
     <tableColumn id="6" name="Punto en que se aprobó"/>
@@ -853,35 +841,35 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>1. Cuerpos: un renglón por cada cuerpo colegiado. Ya vienen el Directorio del FIAS, la Junta Administrativa del FAP y el Directorio del FEIG; se pueden añadir más.</t>
+          <t>1. Fondos: el FIAS y cada fondo, programa o proyecto que administra. Ya vienen FIAS, FAP y FEIG; se añade un renglón por cada otro.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>2. Programas: un renglón por cada programa o proyecto. Con ellos se llena la columna «Programa o proyecto» de Actas y Resoluciones, y así se puede consultar todo lo de un proyecto junto. Si algo es general (no es de ningún proyecto), esa columna se deja vacía.</t>
+          <t>2. Cuerpos: un renglón por cada cuerpo colegiado, con el fondo al que pertenece: la Junta Administrativa del FAP es del FAP. Así, todas sus actas y resoluciones quedan en el FAP sin escribirlo en cada renglón, y en Quórum se consulta cada fondo por separado (o todo junto).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>3. Actas: un renglón por sesión. Cuerpo + fecha de la sesión identifican al acta. Si la sesión trata de uno o varios programas o proyectos, se escriben en «Programa o proyecto», separados con punto y coma. Mientras no tenga enlace al acta definitiva ni fecha de aprobación, se muestra como provisional.</t>
+          <t>3. Actas: un renglón por sesión, de cualquier cuerpo y cualquier fondo, en la misma hoja. Cuerpo + fecha de la sesión identifican al acta. Mientras no tenga enlace al acta definitiva ni fecha de aprobación, se muestra como provisional.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>4. Resoluciones: un renglón por cada punto en que se resolvió algo. Cuerpo + fecha + punto la identifican: «en la Junta Administrativa del 8 de agosto de 2026, en el tercer punto» se escribe JA-FAP · 08/08/2026 · 3. Por omisión es del programa o proyecto de su acta; la columna de programa solo se llena si trata de otro.</t>
+          <t>4. Resoluciones: un renglón por cada punto en que se resolvió algo. Cuerpo + fecha + punto la identifican: «en la Junta Administrativa del 8 de agosto de 2026, en el tercer punto» se escribe JA-FAP · 08/08/2026 · 3.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>5. Normativa: un renglón por norma, con el órgano que la aprueba y la fecha (y si se sabe, el punto) en que se aprobó.</t>
+          <t>5. Normativa: un renglón por norma, con el órgano que la aprueba y la fecha (y si se sabe, el punto) en que se aprobó. Su fondo es el del órgano, salvo que se escriba otro.</t>
         </is>
       </c>
     </row>
@@ -994,14 +982,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="46" customHeight="1">
@@ -1017,15 +1004,10 @@
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>Entidad</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>Grupo de acceso</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -1034,76 +1016,79 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DIR-FIAS</t>
+          <t>FIAS</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Directorio del FIAS</t>
+          <t>Fondo de Inversión Ambiental Sostenible</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>FIAS</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>legal</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="n"/>
+          <t>Institución</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>JA-FAP</t>
+          <t>FAP</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Junta Administrativa del FAP</t>
+          <t>Fondo de Áreas Protegidas</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FAP</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>legal</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="n"/>
+          <t>Fondo</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DIR-FEIG</t>
+          <t>FEIG</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Directorio del FEIG</t>
+          <t>Fondo para el Control de Especies Invasoras de Galápagos</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>FEIG</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>legal</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="n"/>
+          <t>Fondo</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PPD</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Programa de Pequeñas Donaciones</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="C2:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor de la lista" error="Elige un valor de la lista. Si es un cuerpo o una norma nueva, añádelo primero en su hoja." type="list">
-      <formula1>Listas!$A$2:$A$4</formula1>
+      <formula1>Listas!$B$2:$B$5</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1120,82 +1105,98 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="46" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Programa o proyecto</t>
+          <t>Sigla</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
-          <t>Tipo</t>
+          <t>Nombre completo</t>
         </is>
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>Entidad</t>
+          <t>Fondo</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
+          <t>Grupo de acceso</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
           <t>Observaciones</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Programa de Pequeñas Donaciones</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Programa</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DIR-FIAS</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Directorio del FIAS</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>FIAS</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>legal</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>JA-FAP</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Junta Administrativa del FAP</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>FAP</t>
         </is>
       </c>
-      <c r="D2" s="3" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Programa de Gestión de Áreas Protegidas</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>FAP</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="n"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>legal</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Proyecto de Monitoreo de Especies</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Proyecto</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DIR-FEIG</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Directorio del FEIG</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1203,15 +1204,40 @@
           <t>FEIG</t>
         </is>
       </c>
-      <c r="D4" s="3" t="n"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>legal</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CD-PPD</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Comité Directivo del Programa de Pequeñas Donaciones</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PPD</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>legal</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="B2:B2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor de la lista" error="Elige un valor de la lista. Si es un cuerpo o una norma nueva, añádelo primero en su hoja." type="list">
-      <formula1>Listas!$C$2:$C$3</formula1>
-    </dataValidation>
+  <dataValidations count="1">
     <dataValidation sqref="C2:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor de la lista" error="Elige un valor de la lista. Si es un cuerpo o una norma nueva, añádelo primero en su hoja." type="list">
-      <formula1>Listas!$A$2:$A$4</formula1>
+      <formula1>Fondos!$A$2:$A$2000</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1228,7 +1254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1237,9 +1263,8 @@
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="34" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="46" customHeight="1">
@@ -1265,25 +1290,20 @@
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>Programa o proyecto</t>
+          <t>Acta provisional (enlace)</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>Acta provisional (enlace)</t>
+          <t>Acta definitiva (enlace)</t>
         </is>
       </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
-          <t>Acta definitiva (enlace)</t>
+          <t>Fecha de aprobación del acta definitiva</t>
         </is>
       </c>
       <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>Fecha de aprobación del acta definitiva</t>
-        </is>
-      </c>
-      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -1303,20 +1323,20 @@
           <t>Ordinaria</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2017-05-18-provisional.pdf</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2017-05-18-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/DIR-FIAS/2017-05-18-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H2" s="6" t="n">
+      <c r="G2" s="6" t="n">
         <v>43062</v>
       </c>
-      <c r="I2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1332,20 +1352,20 @@
           <t>Ordinaria</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2017-11-23-provisional.pdf</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2017-11-23-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/DIR-FIAS/2017-11-23-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H3" s="6" t="n">
+      <c r="G3" s="6" t="n">
         <v>43328</v>
       </c>
-      <c r="I3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1361,20 +1381,20 @@
           <t>Ordinaria</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2018-08-16-provisional.pdf</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2018-08-16-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/DIR-FIAS/2018-08-16-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H4" s="6" t="n">
+      <c r="G4" s="6" t="n">
         <v>43538</v>
       </c>
-      <c r="I4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1390,20 +1410,20 @@
           <t>Ordinaria</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2019-03-14-provisional.pdf</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2019-03-14-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/DIR-FIAS/2019-03-14-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="G5" s="6" t="n">
         <v>43657</v>
       </c>
-      <c r="I5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1419,20 +1439,20 @@
           <t>Ordinaria</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2019-07-11-provisional.pdf</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2019-07-11-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/DIR-FIAS/2019-07-11-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="G6" s="6" t="n">
         <v>43811</v>
       </c>
-      <c r="I6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1448,20 +1468,20 @@
           <t>Ordinaria</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2019-12-12-provisional.pdf</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2019-12-12-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/DIR-FIAS/2019-12-12-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="G7" s="6" t="n">
         <v>44273</v>
       </c>
-      <c r="I7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1477,20 +1497,20 @@
           <t>Ordinaria</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2021-03-18-provisional.pdf</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2021-03-18-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/DIR-FIAS/2021-03-18-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H8" s="6" t="n">
+      <c r="G8" s="6" t="n">
         <v>44721</v>
       </c>
-      <c r="I8" s="3" t="n"/>
+      <c r="H8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1506,20 +1526,20 @@
           <t>Ordinaria</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2022-06-09-provisional.pdf</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2022-06-09-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/DIR-FIAS/2022-06-09-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H9" s="6" t="n">
+      <c r="G9" s="6" t="n">
         <v>45036</v>
       </c>
-      <c r="I9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1535,20 +1555,20 @@
           <t>Extraordinaria</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2023-04-20-provisional.pdf</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2023-04-20-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/DIR-FIAS/2023-04-20-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H10" s="6" t="n">
+      <c r="G10" s="6" t="n">
         <v>45316</v>
       </c>
-      <c r="I10" s="3" t="n"/>
+      <c r="H10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1564,20 +1584,20 @@
           <t>Ordinaria</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2024-01-25-provisional.pdf</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2024-01-25-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/DIR-FIAS/2024-01-25-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="G11" s="6" t="n">
         <v>45582</v>
       </c>
-      <c r="I11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1593,20 +1613,20 @@
           <t>Ordinaria</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2024-10-17-provisional.pdf</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2024-10-17-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/DIR-FIAS/2024-10-17-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="G12" s="6" t="n">
         <v>45736</v>
       </c>
-      <c r="I12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1622,20 +1642,20 @@
           <t>Ordinaria</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2025-03-20-provisional.pdf</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2025-03-20-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/DIR-FIAS/2025-03-20-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="G13" s="6" t="n">
         <v>45981</v>
       </c>
-      <c r="I13" s="3" t="n"/>
+      <c r="H13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1651,20 +1671,20 @@
           <t>Ordinaria</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2025-11-20-provisional.pdf</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/DIR-FIAS/2025-11-20-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/DIR-FIAS/2025-11-20-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="G14" s="6" t="n">
         <v>46282</v>
       </c>
-      <c r="I14" s="3" t="n"/>
+      <c r="H14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1680,13 +1700,13 @@
           <t>Ordinaria</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>https://ejemplo.invalid/quorum/DIR-FIAS/2026-09-17-provisional.pdf</t>
         </is>
       </c>
-      <c r="H15" s="6" t="n"/>
-      <c r="I15" s="3" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1702,20 +1722,20 @@
           <t>Ordinaria</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/JA-FAP/2017-03-09-provisional.pdf</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/JA-FAP/2017-03-09-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/JA-FAP/2017-03-09-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H16" s="6" t="n">
+      <c r="G16" s="6" t="n">
         <v>43151</v>
       </c>
-      <c r="I16" s="3" t="n"/>
+      <c r="H16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1731,20 +1751,20 @@
           <t>Ordinaria</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/JA-FAP/2018-02-20-provisional.pdf</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/JA-FAP/2018-02-20-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/JA-FAP/2018-02-20-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H17" s="6" t="n">
+      <c r="G17" s="6" t="n">
         <v>44084</v>
       </c>
-      <c r="I17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1760,20 +1780,20 @@
           <t>Ordinaria</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/JA-FAP/2020-09-10-provisional.pdf</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/JA-FAP/2020-09-10-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/JA-FAP/2020-09-10-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H18" s="6" t="n">
+      <c r="G18" s="6" t="n">
         <v>44420</v>
       </c>
-      <c r="I18" s="3" t="n"/>
+      <c r="H18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1789,20 +1809,20 @@
           <t>Ordinaria</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/JA-FAP/2021-08-12-provisional.pdf</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/JA-FAP/2021-08-12-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/JA-FAP/2021-08-12-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H19" s="6" t="n">
+      <c r="G19" s="6" t="n">
         <v>45456</v>
       </c>
-      <c r="I19" s="3" t="n"/>
+      <c r="H19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1820,23 +1840,18 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Programa de Pequeñas Donaciones</t>
+          <t>https://ejemplo.invalid/quorum/JA-FAP/2024-06-13-provisional.pdf</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/JA-FAP/2024-06-13-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/JA-FAP/2024-06-13-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H20" s="6" t="n">
+      <c r="G20" s="6" t="n">
         <v>45547</v>
       </c>
-      <c r="I20" s="3" t="n"/>
+      <c r="H20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1854,23 +1869,18 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Programa de Pequeñas Donaciones</t>
+          <t>https://ejemplo.invalid/quorum/JA-FAP/2024-09-12-provisional.pdf</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/JA-FAP/2024-09-12-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/JA-FAP/2024-09-12-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H21" s="6" t="n">
+      <c r="G21" s="6" t="n">
         <v>46242</v>
       </c>
-      <c r="I21" s="3" t="n"/>
+      <c r="H21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1888,23 +1898,18 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Programa de Pequeñas Donaciones; Programa de Gestión de Áreas Protegidas</t>
+          <t>https://ejemplo.invalid/quorum/JA-FAP/2026-08-08-provisional.pdf</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/JA-FAP/2026-08-08-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/JA-FAP/2026-08-08-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H22" s="6" t="n">
+      <c r="G22" s="6" t="n">
         <v>46296</v>
       </c>
-      <c r="I22" s="3" t="n"/>
+      <c r="H22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1920,13 +1925,13 @@
           <t>Ordinaria</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>https://ejemplo.invalid/quorum/JA-FAP/2026-10-01-provisional.pdf</t>
         </is>
       </c>
-      <c r="H23" s="6" t="n"/>
-      <c r="I23" s="3" t="n"/>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1942,20 +1947,20 @@
           <t>Ordinaria</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/DIR-FEIG/2020-02-13-provisional.pdf</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/DIR-FEIG/2020-02-13-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/DIR-FEIG/2020-02-13-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H24" s="6" t="n">
+      <c r="G24" s="6" t="n">
         <v>45792</v>
       </c>
-      <c r="I24" s="3" t="n"/>
+      <c r="H24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1971,20 +1976,20 @@
           <t>Ordinaria</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/DIR-FEIG/2025-05-15-provisional.pdf</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://ejemplo.invalid/quorum/DIR-FEIG/2025-05-15-provisional.pdf</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
           <t>https://ejemplo.invalid/quorum/DIR-FEIG/2025-05-15-definitiva.pdf</t>
         </is>
       </c>
-      <c r="H25" s="6" t="n">
+      <c r="G25" s="6" t="n">
         <v>46156</v>
       </c>
-      <c r="I25" s="3" t="n"/>
+      <c r="H25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2000,13 +2005,64 @@
           <t>Ordinaria</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>https://ejemplo.invalid/quorum/DIR-FEIG/2026-05-14-provisional.pdf</t>
         </is>
       </c>
-      <c r="H26" s="6" t="n"/>
-      <c r="I26" s="3" t="n"/>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" s="3" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CD-PPD</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="n">
+        <v>45699</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Ordinaria</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/CD-PPD/2025-02-11-provisional.pdf</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/CD-PPD/2025-02-11-definitiva.pdf</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>45909</v>
+      </c>
+      <c r="H27" s="3" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CD-PPD</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="n">
+        <v>45909</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Ordinaria</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://ejemplo.invalid/quorum/CD-PPD/2025-09-09-provisional.pdf</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="n"/>
+      <c r="H28" s="3" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="4">
@@ -2017,9 +2073,9 @@
       <formula1>DATE(1990,1,1)</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor de la lista" error="Elige un valor de la lista. Si es un cuerpo o una norma nueva, añádelo primero en su hoja." type="list">
-      <formula1>Listas!$B$2:$B$3</formula1>
+      <formula1>Listas!$A$2:$A$3</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fecha" error="Escribe una fecha: dd/mm/aaaa." type="date" operator="greaterThan">
+    <dataValidation sqref="G2:G2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fecha" error="Escribe una fecha: dd/mm/aaaa." type="date" operator="greaterThan">
       <formula1>DATE(1990,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -2037,7 +2093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2045,9 +2101,8 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="46" customHeight="1">
@@ -2078,15 +2133,10 @@
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>Programa o proyecto (solo si es distinto del acta)</t>
+          <t>Enlace (opcional)</t>
         </is>
       </c>
       <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>Enlace (opcional)</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -2116,7 +2166,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2142,7 +2192,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2168,7 +2218,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H4" s="3" t="n"/>
+      <c r="G4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2194,7 +2244,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2220,7 +2270,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H6" s="3" t="n"/>
+      <c r="G6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2246,7 +2296,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2272,7 +2322,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H8" s="3" t="n"/>
+      <c r="G8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2298,7 +2348,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2324,7 +2374,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H10" s="3" t="n"/>
+      <c r="G10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2350,7 +2400,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2376,7 +2426,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H12" s="3" t="n"/>
+      <c r="G12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2402,7 +2452,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H13" s="3" t="n"/>
+      <c r="G13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2428,7 +2478,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H14" s="3" t="n"/>
+      <c r="G14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2454,7 +2504,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H15" s="3" t="n"/>
+      <c r="G15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2480,7 +2530,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H16" s="3" t="n"/>
+      <c r="G16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2506,7 +2556,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H17" s="3" t="n"/>
+      <c r="G17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2532,7 +2582,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H18" s="3" t="n"/>
+      <c r="G18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2558,7 +2608,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H19" s="3" t="n"/>
+      <c r="G19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2584,7 +2634,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H20" s="3" t="n"/>
+      <c r="G20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2610,7 +2660,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H21" s="3" t="n"/>
+      <c r="G21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2636,7 +2686,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H22" s="3" t="n"/>
+      <c r="G22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2662,25 +2712,25 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H23" s="3" t="n"/>
+      <c r="G23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>DIR-FIAS</t>
+          <t>CD-PPD</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>42873</v>
+        <v>45909</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Conocer y aprobar el informe de gestión del primer trimestre de 2017.</t>
+          <t>Aprobar el acta de la sesión del 11/02/2025.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2688,7 +2738,7 @@
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H24" s="3" t="n"/>
+      <c r="G24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2701,20 +2751,20 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Aprobar el Reglamento de Adquisiciones del FIAS.</t>
+          <t>Conocer y aprobar el informe de gestión del primer trimestre de 2017.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Normativa</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="n"/>
+          <t>Gobierno corporativo</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2723,24 +2773,24 @@
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>43062</v>
+        <v>42873</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Aprobar la Política de Inversiones del FIAS.</t>
+          <t>Aprobar el Reglamento de Adquisiciones del FIAS.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Inversiones</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="n"/>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2753,20 +2803,20 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Aprobar el presupuesto institucional 2018.</t>
+          <t>Aprobar la Política de Inversiones del FIAS.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Presupuesto y finanzas</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="n"/>
+          <t>Inversiones</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2775,7 +2825,7 @@
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>43328</v>
+        <v>43062</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -2784,15 +2834,15 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Designar al auditor externo para el ejercicio 2018.</t>
+          <t>Aprobar el presupuesto institucional 2018.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Designaciones</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="n"/>
+          <t>Presupuesto y finanzas</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2805,20 +2855,20 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Aprobar el Código de Ética y Conducta del FIAS.</t>
+          <t>Designar al auditor externo para el ejercicio 2018.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Normativa</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="n"/>
+          <t>Designaciones</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2827,16 +2877,16 @@
         </is>
       </c>
       <c r="B30" s="6" t="n">
-        <v>43538</v>
+        <v>43328</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Reformar los artículos 12 y 15 del Reglamento de Adquisiciones para actualizar los montos de contratación directa.</t>
+          <t>Aprobar el Código de Ética y Conducta del FIAS.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2844,7 +2894,7 @@
           <t>Normativa</t>
         </is>
       </c>
-      <c r="H30" s="3" t="n"/>
+      <c r="G30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2853,24 +2903,24 @@
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>43657</v>
+        <v>43538</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Aprobar el Reglamento Interno de Talento Humano.</t>
+          <t>Reformar los artículos 12 y 15 del Reglamento de Adquisiciones para actualizar los montos de contratación directa.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Talento humano</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="n"/>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2879,24 +2929,24 @@
         </is>
       </c>
       <c r="B32" s="6" t="n">
-        <v>43811</v>
+        <v>43657</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Aprobar el presupuesto institucional 2020.</t>
+          <t>Aprobar el Reglamento Interno de Talento Humano.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Presupuesto y finanzas</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="n"/>
+          <t>Talento humano</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2909,20 +2959,20 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Aprobar el Procedimiento de Viáticos y Movilización.</t>
+          <t>Aprobar el presupuesto institucional 2020.</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Normativa</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="n"/>
+          <t>Presupuesto y finanzas</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2931,24 +2981,24 @@
         </is>
       </c>
       <c r="B34" s="6" t="n">
-        <v>44273</v>
+        <v>43811</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Aprobar los Lineamientos de Teletrabajo.</t>
+          <t>Aprobar el Procedimiento de Viáticos y Movilización.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Talento humano</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="n"/>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2957,24 +3007,24 @@
         </is>
       </c>
       <c r="B35" s="6" t="n">
-        <v>44721</v>
+        <v>44273</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Aprobar la codificación del Reglamento de Adquisiciones del FIAS, que integra sus reformas.</t>
+          <t>Aprobar los Lineamientos de Teletrabajo.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Normativa</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="n"/>
+          <t>Talento humano</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2983,24 +3033,24 @@
         </is>
       </c>
       <c r="B36" s="6" t="n">
-        <v>45036</v>
+        <v>44721</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Aprobar la Política de Inversiones y Gestión de Portafolio y derogar la Política de Inversiones de 2017.</t>
+          <t>Aprobar la codificación del Reglamento de Adquisiciones del FIAS, que integra sus reformas.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Inversiones</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="n"/>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3009,24 +3059,24 @@
         </is>
       </c>
       <c r="B37" s="6" t="n">
-        <v>45316</v>
+        <v>45036</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Reformar el capítulo V del Reglamento Interno de Talento Humano para integrar el régimen de viáticos.</t>
+          <t>Aprobar la Política de Inversiones y Gestión de Portafolio y derogar la Política de Inversiones de 2017.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Talento humano</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="n"/>
+          <t>Inversiones</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3039,20 +3089,20 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Derogar el Procedimiento de Viáticos y Movilización, cuyo contenido pasa al Reglamento Interno de Talento Humano.</t>
+          <t>Reformar el capítulo V del Reglamento Interno de Talento Humano para integrar el régimen de viáticos.</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Normativa</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="n"/>
+          <t>Talento humano</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3061,24 +3111,24 @@
         </is>
       </c>
       <c r="B39" s="6" t="n">
-        <v>45582</v>
+        <v>45316</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Aclarar el alcance del artículo 8 de la Política de Inversiones y Gestión de Portafolio sobre los límites por emisor.</t>
+          <t>Derogar el Procedimiento de Viáticos y Movilización, cuyo contenido pasa al Reglamento Interno de Talento Humano.</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Inversiones</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="n"/>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3087,24 +3137,24 @@
         </is>
       </c>
       <c r="B40" s="6" t="n">
-        <v>45736</v>
+        <v>45582</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Designar a la Gerencia Financiera como representante del FIAS ante el comité de inversiones.</t>
+          <t>Aclarar el alcance del artículo 8 de la Política de Inversiones y Gestión de Portafolio sobre los límites por emisor.</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Designaciones</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="n"/>
+          <t>Inversiones</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3113,16 +3163,16 @@
         </is>
       </c>
       <c r="B41" s="6" t="n">
-        <v>45981</v>
+        <v>45736</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Reformar la designación del 20 de marzo de 2025: la representación ante el comité de inversiones la ejerce la Dirección Ejecutiva.</t>
+          <t>Designar a la Gerencia Financiera como representante del FIAS ante el comité de inversiones.</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3130,7 +3180,7 @@
           <t>Designaciones</t>
         </is>
       </c>
-      <c r="H41" s="3" t="n"/>
+      <c r="G41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3139,7 +3189,7 @@
         </is>
       </c>
       <c r="B42" s="6" t="n">
-        <v>46282</v>
+        <v>45981</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -3148,15 +3198,15 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Derogar los Lineamientos de Teletrabajo a partir del 1 de enero de 2027.</t>
+          <t>Reformar la designación del 20 de marzo de 2025: la representación ante el comité de inversiones la ejerce la Dirección Ejecutiva.</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Talento humano</t>
-        </is>
-      </c>
-      <c r="H42" s="3" t="n"/>
+          <t>Designaciones</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3169,29 +3219,29 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Aprobar el presupuesto institucional 2027.</t>
+          <t>Derogar los Lineamientos de Teletrabajo a partir del 1 de enero de 2027.</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Presupuesto y finanzas</t>
-        </is>
-      </c>
-      <c r="H43" s="3" t="n"/>
+          <t>Talento humano</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="n"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>JA-FAP</t>
+          <t>DIR-FIAS</t>
         </is>
       </c>
       <c r="B44" s="6" t="n">
-        <v>42803</v>
+        <v>46282</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -3200,15 +3250,15 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Aprobar el Reglamento de Funcionamiento de la Junta Administrativa del FAP.</t>
+          <t>Aprobar el presupuesto institucional 2027.</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Gobierno corporativo</t>
-        </is>
-      </c>
-      <c r="H44" s="3" t="n"/>
+          <t>Presupuesto y finanzas</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="n"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3217,24 +3267,24 @@
         </is>
       </c>
       <c r="B45" s="6" t="n">
-        <v>43151</v>
+        <v>42803</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Aprobar el Manual Operativo del Ciclo de Proyectos del FAP.</t>
+          <t>Aprobar el Reglamento de Funcionamiento de la Junta Administrativa del FAP.</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Normativa</t>
-        </is>
-      </c>
-      <c r="H45" s="3" t="n"/>
+          <t>Gobierno corporativo</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="n"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3243,24 +3293,24 @@
         </is>
       </c>
       <c r="B46" s="6" t="n">
-        <v>44084</v>
+        <v>43151</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Aprobar la codificación del Reglamento de Funcionamiento de la Junta Administrativa.</t>
+          <t>Aprobar el Manual Operativo del Ciclo de Proyectos del FAP.</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Gobierno corporativo</t>
-        </is>
-      </c>
-      <c r="H46" s="3" t="n"/>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="n"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3269,24 +3319,24 @@
         </is>
       </c>
       <c r="B47" s="6" t="n">
-        <v>44420</v>
+        <v>44084</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Reformar la sección de seguimiento técnico del Manual Operativo del Ciclo de Proyectos.</t>
+          <t>Aprobar la codificación del Reglamento de Funcionamiento de la Junta Administrativa.</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Normativa</t>
-        </is>
-      </c>
-      <c r="H47" s="3" t="n"/>
+          <t>Gobierno corporativo</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3295,24 +3345,24 @@
         </is>
       </c>
       <c r="B48" s="6" t="n">
-        <v>45456</v>
+        <v>44420</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Aprobar las bases de la convocatoria de pequeñas donaciones 2024, con cierre el 30 de septiembre.</t>
+          <t>Reformar la sección de seguimiento técnico del Manual Operativo del Ciclo de Proyectos.</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Proyectos y convocatorias</t>
-        </is>
-      </c>
-      <c r="H48" s="3" t="n"/>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="n"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3321,16 +3371,16 @@
         </is>
       </c>
       <c r="B49" s="6" t="n">
-        <v>45547</v>
+        <v>45456</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Dejar sin efecto la convocatoria de pequeñas donaciones 2024 por falta de disponibilidad presupuestaria.</t>
+          <t>Aprobar las bases de la convocatoria de pequeñas donaciones 2024, con cierre el 30 de septiembre.</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -3338,7 +3388,7 @@
           <t>Proyectos y convocatorias</t>
         </is>
       </c>
-      <c r="H49" s="3" t="n"/>
+      <c r="G49" s="3" t="n"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3347,24 +3397,24 @@
         </is>
       </c>
       <c r="B50" s="6" t="n">
-        <v>46242</v>
+        <v>45547</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Aprobar la reforma integral del Manual Operativo del Ciclo de Proyectos del FAP.</t>
+          <t>Dejar sin efecto la convocatoria de pequeñas donaciones 2024 por falta de disponibilidad presupuestaria.</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Normativa</t>
-        </is>
-      </c>
-      <c r="H50" s="3" t="n"/>
+          <t>Proyectos y convocatorias</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="n"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3377,25 +3427,20 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Aprobar el plan operativo anual 2027 de las áreas protegidas.</t>
+          <t>Aprobar la reforma integral del Manual Operativo del Ciclo de Proyectos del FAP.</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Presupuesto y finanzas</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>Programa de Gestión de Áreas Protegidas</t>
-        </is>
-      </c>
-      <c r="H51" s="3" t="n"/>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="n"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3404,50 +3449,50 @@
         </is>
       </c>
       <c r="B52" s="6" t="n">
-        <v>46296</v>
+        <v>46242</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Conocer el informe de avance de la campaña de renovaciones 2027.</t>
+          <t>Aprobar el plan operativo anual 2027 de las áreas protegidas.</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Administrativo</t>
-        </is>
-      </c>
-      <c r="H52" s="3" t="n"/>
+          <t>Presupuesto y finanzas</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="n"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>DIR-FEIG</t>
+          <t>JA-FAP</t>
         </is>
       </c>
       <c r="B53" s="6" t="n">
-        <v>43874</v>
+        <v>46296</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Aprobar el Manual de Operaciones del FEIG.</t>
+          <t>Conocer el informe de avance de la campaña de renovaciones 2027.</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Normativa</t>
-        </is>
-      </c>
-      <c r="H53" s="3" t="n"/>
+          <t>Administrativo</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="n"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3456,16 +3501,16 @@
         </is>
       </c>
       <c r="B54" s="6" t="n">
-        <v>45792</v>
+        <v>43874</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Reformar el Manual de Operaciones del FEIG para incorporar los desembolsos por hitos, desde el 1 de julio de 2025.</t>
+          <t>Aprobar el Manual de Operaciones del FEIG.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -3473,7 +3518,7 @@
           <t>Normativa</t>
         </is>
       </c>
-      <c r="H54" s="3" t="n"/>
+      <c r="G54" s="3" t="n"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3482,7 +3527,7 @@
         </is>
       </c>
       <c r="B55" s="6" t="n">
-        <v>46156</v>
+        <v>45792</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -3491,15 +3536,15 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Aprobar el informe financiero del primer trimestre de 2026.</t>
+          <t>Reformar el Manual de Operaciones del FEIG para incorporar los desembolsos por hitos, desde el 1 de julio de 2025.</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Presupuesto y finanzas</t>
-        </is>
-      </c>
-      <c r="H55" s="3" t="n"/>
+          <t>Normativa</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="n"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3512,25 +3557,20 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Aprobar el convenio de cooperación con una universidad para el monitoreo de especies.</t>
+          <t>Aprobar el informe financiero del primer trimestre de 2026.</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Convenios y alianzas</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>Proyecto de Monitoreo de Especies</t>
-        </is>
-      </c>
-      <c r="H56" s="3" t="n"/>
+          <t>Presupuesto y finanzas</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="n"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3539,24 +3579,102 @@
         </is>
       </c>
       <c r="B57" s="6" t="n">
+        <v>46156</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Aprobar el convenio de cooperación con una universidad para el monitoreo de especies.</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Convenios y alianzas</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>DIR-FEIG</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="n">
         <v>44875</v>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>Ratificar la integración del comité técnico del FEIG.</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E58" t="inlineStr">
         <is>
           <t>Gobierno corporativo</t>
         </is>
       </c>
-      <c r="H57" s="3" t="n"/>
+      <c r="G58" s="3" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>CD-PPD</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="n">
+        <v>45699</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Aprobar el plan de trabajo 2025 del programa.</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Proyectos y convocatorias</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>CD-PPD</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="n">
+        <v>45909</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Seleccionar los proyectos ganadores de la convocatoria 2025.</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Proyectos y convocatorias</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -3567,7 +3685,7 @@
       <formula1>DATE(1990,1,1)</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor de la lista" error="Elige un valor de la lista. Si es un cuerpo o una norma nueva, añádelo primero en su hoja." type="list">
-      <formula1>Listas!$E$2:$E$11</formula1>
+      <formula1>Listas!$D$2:$D$11</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3611,7 +3729,7 @@
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>Entidad</t>
+          <t>Fondo</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">
@@ -4008,10 +4126,10 @@
   </sheetData>
   <dataValidations count="4">
     <dataValidation sqref="B2:B2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor de la lista" error="Elige un valor de la lista. Si es un cuerpo o una norma nueva, añádelo primero en su hoja." type="list">
-      <formula1>Listas!$D$2:$D$10</formula1>
+      <formula1>Listas!$C$2:$C$10</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor de la lista" error="Elige un valor de la lista. Si es un cuerpo o una norma nueva, añádelo primero en su hoja." type="list">
-      <formula1>Listas!$A$2:$A$4</formula1>
+      <formula1>Fondos!$A$2:$A$2000</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor de la lista" error="Elige un valor de la lista. Si es un cuerpo o una norma nueva, añádelo primero en su hoja." type="list">
       <formula1>Cuerpos!$A$2:$A$2000</formula1>
@@ -4567,7 +4685,7 @@
       <formula1>DATE(1990,1,1)</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor de la lista" error="Elige un valor de la lista. Si es un cuerpo o una norma nueva, añádelo primero en su hoja." type="list">
-      <formula1>Listas!$F$2:$F$7</formula1>
+      <formula1>Listas!$E$2:$E$7</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor de la lista" error="Elige un valor de la lista. Si es un cuerpo o una norma nueva, añádelo primero en su hoja." type="list">
       <formula1>Cuerpos!$A$2:$A$2000</formula1>
@@ -4593,7 +4711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4601,36 +4719,30 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>ENTIDADES</t>
+          <t>TIPOS_SESION</t>
         </is>
       </c>
       <c r="B1" s="7" t="inlineStr">
         <is>
-          <t>TIPOS_SESION</t>
+          <t>TIPOS_FONDO</t>
         </is>
       </c>
       <c r="C1" s="7" t="inlineStr">
         <is>
-          <t>TIPOS_PROG</t>
+          <t>TIPOS_NORMA</t>
         </is>
       </c>
       <c r="D1" s="7" t="inlineStr">
         <is>
-          <t>TIPOS_NORMA</t>
+          <t>MATERIAS</t>
         </is>
       </c>
       <c r="E1" s="7" t="inlineStr">
-        <is>
-          <t>MATERIAS</t>
-        </is>
-      </c>
-      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>TIPOS_CAMBIO</t>
         </is>
@@ -4639,30 +4751,25 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FIAS</t>
+          <t>Ordinaria</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ordinaria</t>
+          <t>Institución</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Programa</t>
+          <t>Estatuto</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Estatuto</t>
+          <t>Normativa</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
-        <is>
-          <t>Normativa</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
         <is>
           <t>Reforma</t>
         </is>
@@ -4671,146 +4778,146 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FAP</t>
+          <t>Extraordinaria</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Extraordinaria</t>
+          <t>Fondo</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Reglamento</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Presupuesto y finanzas</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Reforma parcial</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Inversiones</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Codificación</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
           <t>Proyecto</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Reglamento</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Presupuesto y finanzas</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Reforma parcial</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>FEIG</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Inversiones</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Codificación</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Política</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Política</t>
+          <t>Proyectos y convocatorias</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Proyectos y convocatorias</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
           <t>Derogación</t>
         </is>
       </c>
     </row>
     <row r="6">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Procedimiento</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Procedimiento</t>
+          <t>Convenios y alianzas</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Convenios y alianzas</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
           <t>Deja sin efecto</t>
         </is>
       </c>
     </row>
     <row r="7">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Instructivo</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Instructivo</t>
+          <t>Talento humano</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Talento humano</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
           <t>Aclaración</t>
         </is>
       </c>
     </row>
     <row r="8">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Lineamiento</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Lineamiento</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
           <t>Designaciones</t>
         </is>
       </c>
     </row>
     <row r="9">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Código</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
           <t>Gobierno corporativo</t>
         </is>
       </c>
     </row>
     <row r="10">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Otro</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Otro</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
           <t>Administrativo</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="E11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Otros</t>
         </is>

</xml_diff>